<commit_message>
análisis: hoja Ref+Subestación agrupada por cambio de troncal
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PkC9T9h9bWvat77XCKHKnu
</commit_message>
<xml_diff>
--- a/docs/precio_por_barra_criterios.xlsx
+++ b/docs/precio_por_barra_criterios.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referido + Subestación vs PN260" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ref+Subestación vs PN2604" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referido vs PN2604" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Módulo actual vs PN2604" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ref+Sub por cambio" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,7 +515,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Referido + Subestación vs PN2604</t>
+          <t>Ref+Subestación vs PN2604</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -541,7 +542,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Referido + Subestación vs PN2604</t>
+          <t>Ref+Subestación vs PN2604</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -55576,4 +55577,1782 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="37" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Barras</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Con PSUF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Δ precio ($/kW/mes)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>km entre troncales</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Inyección (MW)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Retiro (MW)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Flujo Tx (MW)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Monto iny+ret (MM$/mes)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Monto si Tx se valorizara (MM$/mes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C.CHENA → A.JAHUEL</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-247.7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>21</v>
+      </c>
+      <c r="F2" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>365.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1462.7</v>
+      </c>
+      <c r="I2" t="n">
+        <v>95</v>
+      </c>
+      <c r="J2" t="n">
+        <v>362.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CANDELARIA → A.JAHUEL</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3" t="n">
+        <v>492</v>
+      </c>
+      <c r="E3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F3" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>166.2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>523.7</v>
+      </c>
+      <c r="I3" t="n">
+        <v>93.3</v>
+      </c>
+      <c r="J3" t="n">
+        <v>257.7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>QUILLOTA → NOGALES</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>39</v>
+      </c>
+      <c r="C4" t="n">
+        <v>36</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-187.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>26</v>
+      </c>
+      <c r="F4" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>401.7</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1097.9</v>
+      </c>
+      <c r="I4" t="n">
+        <v>85.8</v>
+      </c>
+      <c r="J4" t="n">
+        <v>205.9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CAUTIN → CIRUELOS</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1730.6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>97</v>
+      </c>
+      <c r="F5" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>233.5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="J5" t="n">
+        <v>404.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CRUCERO → LAGUNAS</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>215</v>
+      </c>
+      <c r="E6" t="n">
+        <v>163</v>
+      </c>
+      <c r="F6" t="n">
+        <v>140</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>356.6</v>
+      </c>
+      <c r="I6" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>76.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ATACAMA → OHIGGINS</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-232.2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>70</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G7" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="H7" t="n">
+        <v>144.7</v>
+      </c>
+      <c r="I7" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="J7" t="n">
+        <v>33.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CHARRUA → CAUTIN</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-452.4</v>
+      </c>
+      <c r="E8" t="n">
+        <v>182</v>
+      </c>
+      <c r="F8" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>299.9</v>
+      </c>
+      <c r="I8" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="J8" t="n">
+        <v>135.7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P.AZUCAR → L.VILOS</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>295.9</v>
+      </c>
+      <c r="E9" t="n">
+        <v>219</v>
+      </c>
+      <c r="F9" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>29.9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NOGALES → QUILLOTA</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" t="n">
+        <v>187.5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>26</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>99.7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>18.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ATACAMA → LABERINTO</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-281.2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>110</v>
+      </c>
+      <c r="F11" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>68</v>
+      </c>
+      <c r="I11" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="J11" t="n">
+        <v>19.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ATACAMA → CANDELARIA</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-812.8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1217</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="H12" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="I12" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="J12" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RAHUE → TEMUCO</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-1567.8</v>
+      </c>
+      <c r="E13" t="n">
+        <v>212</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="J13" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C.CHENA → C.NAVIA</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>30</v>
+      </c>
+      <c r="C14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>12</v>
+      </c>
+      <c r="F14" t="n">
+        <v>67</v>
+      </c>
+      <c r="G14" t="n">
+        <v>655.5</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2332</v>
+      </c>
+      <c r="I14" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="J14" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OHIGGINS → ATACAMA</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>232.2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>70</v>
+      </c>
+      <c r="F15" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="H15" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="I15" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="J15" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>QUILLOTA → A.MELIP</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>25</v>
+      </c>
+      <c r="C16" t="n">
+        <v>25</v>
+      </c>
+      <c r="D16" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>82</v>
+      </c>
+      <c r="F16" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="H16" t="n">
+        <v>498.5</v>
+      </c>
+      <c r="I16" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="J16" t="n">
+        <v>51.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CHARRUA → OHIGGINS</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1331.4</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1504</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="J17" t="n">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NOGALES → L.VILOS</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>201.2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>90</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G18" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="H18" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J18" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>D.ALMAGRO → C.PINTO</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-31.8</v>
+      </c>
+      <c r="E19" t="n">
+        <v>68</v>
+      </c>
+      <c r="F19" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>364.7</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J19" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>D.ALMAGRO → CARDONES</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="E20" t="n">
+        <v>126</v>
+      </c>
+      <c r="F20" t="n">
+        <v>104</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2110</v>
+      </c>
+      <c r="I20" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="J20" t="n">
+        <v>58.2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NOGALES → L.MAQUIS</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>196.1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>78</v>
+      </c>
+      <c r="F21" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G21" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RAHUE → MELIPULLI</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-205.4</v>
+      </c>
+      <c r="E22" t="n">
+        <v>98</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H22" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J22" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ITAHUE → CANDELARIA</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>707</v>
+      </c>
+      <c r="E23" t="n">
+        <v>141</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>P.COLORADA → MAITENCILLO</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-39.5</v>
+      </c>
+      <c r="E24" t="n">
+        <v>93</v>
+      </c>
+      <c r="F24" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="I24" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J24" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ITAHUE → ANCOA</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" t="n">
+        <v>7</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-116.1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>60</v>
+      </c>
+      <c r="F25" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="G25" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H25" t="n">
+        <v>174.3</v>
+      </c>
+      <c r="I25" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J25" t="n">
+        <v>20.2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>A.MELIP → RAPEL</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>9</v>
+      </c>
+      <c r="C26" t="n">
+        <v>9</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-50.8</v>
+      </c>
+      <c r="E26" t="n">
+        <v>50</v>
+      </c>
+      <c r="F26" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G26" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="H26" t="n">
+        <v>79.40000000000001</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J26" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RAHUE → VALDIVIA</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-49.9</v>
+      </c>
+      <c r="E27" t="n">
+        <v>86</v>
+      </c>
+      <c r="F27" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="G27" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="H27" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J27" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CHARRUA → RAPEL</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1477.6</v>
+      </c>
+      <c r="E28" t="n">
+        <v>346</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>C.PINTO → CARDONES</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>72</v>
+      </c>
+      <c r="F29" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>241.8</v>
+      </c>
+      <c r="I29" t="n">
+        <v>2</v>
+      </c>
+      <c r="J29" t="n">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>VALDIVIA → CIRUELOS</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="E30" t="n">
+        <v>37</v>
+      </c>
+      <c r="F30" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="G30" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="H30" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>HUALPEN → LAGUNILLAS</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>8</v>
+      </c>
+      <c r="C31" t="n">
+        <v>6</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-11.2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>22</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>36</v>
+      </c>
+      <c r="H31" t="n">
+        <v>115.7</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MAITENCILLO → P.AZUCAR</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="n">
+        <v>134.1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>164</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="H32" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J32" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ANCOA → ITAHUE</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>116.1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>60</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>A.JAHUEL → C.CHENA</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>247.7</v>
+      </c>
+      <c r="E34" t="n">
+        <v>21</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>218.8</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>54.2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>A.JAHUEL → C.NAVIA</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>258</v>
+      </c>
+      <c r="E35" t="n">
+        <v>33</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>459.9</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>118.7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CAUTIN → TEMUCO</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="n">
+        <v>178.9</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>221.1</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>39.6</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CHARRUA → ANCOA</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-72.3</v>
+      </c>
+      <c r="E37" t="n">
+        <v>178</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CARDONES → MAITENCILLO</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-75.7</v>
+      </c>
+      <c r="E38" t="n">
+        <v>128</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>C.NAVIA → A.JAHUEL</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-258</v>
+      </c>
+      <c r="E39" t="n">
+        <v>33</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>802.2</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ELCOBRE → CHARRUA</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-1287.5</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1543</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>25</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>32.2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CHILOE → MELIPULLI</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E41" t="n">
+        <v>99</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ELCOBRE → OHIGGINS</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="E42" t="n">
+        <v>89</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ITAHUE → L.MAQUIS</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1390</v>
+      </c>
+      <c r="E43" t="n">
+        <v>268</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>34.9</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>L.MAQUIS → NOGALES</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-196.1</v>
+      </c>
+      <c r="E44" t="n">
+        <v>78</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>LABERINTO → OHIGGINS</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>49</v>
+      </c>
+      <c r="E45" t="n">
+        <v>87</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>633.6</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ITAHUE → CARDONES</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1040.8</v>
+      </c>
+      <c r="E46" t="n">
+        <v>856</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>P.ALMONTE → PARINACOTA</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>172</v>
+      </c>
+      <c r="E47" t="n">
+        <v>211</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>P.MONTT → MELIPULLI</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>P.AZUCAR → C.NAVIA</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>357.8</v>
+      </c>
+      <c r="E49" t="n">
+        <v>386</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
+        <v>193.3</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="n">
+        <v>69.2</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>QUILLOTA → L.MAQUIS</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="E50" t="n">
+        <v>79</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>QUILLOTA → CHARRUA</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" t="n">
+        <v>-1425.2</v>
+      </c>
+      <c r="E51" t="n">
+        <v>471</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>